<commit_message>
[master] - Add IF NOT EXISTS clause to CREATE TABLE SQL statement
</commit_message>
<xml_diff>
--- a/.claude_cowork/eribe-migration-intake.xlsx
+++ b/.claude_cowork/eribe-migration-intake.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Projects\TypeScript\sluice\.claude_cowork\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00E5A20F-DAF6-458D-925B-499761C493FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5F8CECF-F667-4926-82AD-9055375BE931}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21270" yWindow="-21710" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17310" yWindow="-21710" windowWidth="38620" windowHeight="21100" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INSTRUCTIONS" sheetId="1" r:id="rId1"/>
@@ -1154,16 +1154,19 @@
     <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1197,25 +1200,22 @@
     <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1524,62 +1524,62 @@
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
-    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="2" max="2" width="38.59765625" customWidth="1"/>
     <col min="3" max="3" width="80" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
     </row>
     <row r="2" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
     </row>
     <row r="3" spans="1:3" ht="8" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="4" spans="1:3" ht="62" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B4" s="27" t="s">
+      <c r="B4" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="28" t="s">
+      <c r="C4" s="30" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="62" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="28" t="s">
+      <c r="C6" s="30" t="s">
         <v>275</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="126" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B8" s="27" t="s">
+      <c r="B8" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="28" t="s">
+      <c r="C8" s="30" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="110" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B10" s="27" t="s">
+      <c r="B10" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="28" t="s">
+      <c r="C10" s="30" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="62" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B12" s="27" t="s">
+      <c r="B12" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="28" t="s">
+      <c r="C12" s="30" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1617,26 +1617,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
     </row>
     <row r="2" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
     </row>
     <row r="3" spans="1:4" ht="8" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="4" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B4" s="32" t="s">
+      <c r="B4" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
     </row>
     <row r="5" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B5" s="1" t="s">
@@ -1694,11 +1694,11 @@
     </row>
     <row r="11" spans="1:4" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="12" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B12" s="32" t="s">
+      <c r="B12" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="30"/>
-      <c r="D12" s="30"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="29"/>
     </row>
     <row r="13" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B13" s="1" t="s">
@@ -1719,7 +1719,7 @@
       </c>
     </row>
     <row r="15" spans="1:4" ht="52.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B15" s="48" t="s">
+      <c r="B15" s="27" t="s">
         <v>31</v>
       </c>
       <c r="C15" s="4"/>
@@ -1746,7 +1746,7 @@
       </c>
     </row>
     <row r="18" spans="2:4" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B18" s="48" t="s">
+      <c r="B18" s="27" t="s">
         <v>37</v>
       </c>
       <c r="C18" s="4"/>
@@ -1756,11 +1756,11 @@
     </row>
     <row r="19" spans="2:4" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="20" spans="2:4" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B20" s="32" t="s">
+      <c r="B20" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="C20" s="30"/>
-      <c r="D20" s="30"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
     </row>
     <row r="21" spans="2:4" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B21" s="1" t="s">
@@ -1791,11 +1791,11 @@
     </row>
     <row r="24" spans="2:4" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="25" spans="2:4" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B25" s="32" t="s">
+      <c r="B25" s="33" t="s">
         <v>46</v>
       </c>
-      <c r="C25" s="30"/>
-      <c r="D25" s="30"/>
+      <c r="C25" s="29"/>
+      <c r="D25" s="29"/>
     </row>
     <row r="26" spans="2:4" ht="60" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B26" s="5" t="s">
@@ -1848,18 +1848,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
     </row>
     <row r="2" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
     </row>
     <row r="3" spans="1:9" ht="8" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="4" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.45">
@@ -2140,16 +2140,16 @@
       <c r="I29" s="9"/>
     </row>
     <row r="31" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B31" s="33" t="s">
+      <c r="B31" s="34" t="s">
         <v>59</v>
       </c>
-      <c r="C31" s="30"/>
-      <c r="D31" s="30"/>
-      <c r="E31" s="30"/>
-      <c r="F31" s="30"/>
-      <c r="G31" s="30"/>
-      <c r="H31" s="30"/>
-      <c r="I31" s="30"/>
+      <c r="C31" s="29"/>
+      <c r="D31" s="29"/>
+      <c r="E31" s="29"/>
+      <c r="F31" s="29"/>
+      <c r="G31" s="29"/>
+      <c r="H31" s="29"/>
+      <c r="I31" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2192,35 +2192,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
     </row>
     <row r="2" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="32" t="s">
         <v>61</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
     </row>
     <row r="3" spans="1:13" ht="8" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="4" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B4" s="35" t="s">
+      <c r="B4" s="36" t="s">
         <v>62</v>
       </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
-      <c r="F4" s="30"/>
-      <c r="G4" s="30"/>
-      <c r="H4" s="30"/>
-      <c r="I4" s="30"/>
-      <c r="J4" s="30"/>
-      <c r="K4" s="30"/>
-      <c r="L4" s="30"/>
-      <c r="M4" s="30"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="29"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="29"/>
+      <c r="I4" s="29"/>
+      <c r="J4" s="29"/>
+      <c r="K4" s="29"/>
+      <c r="L4" s="29"/>
+      <c r="M4" s="29"/>
     </row>
     <row r="5" spans="1:13" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="6"/>
@@ -2542,144 +2542,144 @@
       <c r="M25" s="10"/>
     </row>
     <row r="27" spans="2:13" ht="28.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B27" s="33" t="s">
+      <c r="B27" s="34" t="s">
         <v>75</v>
       </c>
-      <c r="C27" s="30"/>
-      <c r="D27" s="30"/>
-      <c r="E27" s="30"/>
-      <c r="F27" s="30"/>
-      <c r="G27" s="30"/>
-      <c r="H27" s="30"/>
-      <c r="I27" s="30"/>
-      <c r="J27" s="30"/>
-      <c r="K27" s="30"/>
-      <c r="L27" s="30"/>
-      <c r="M27" s="30"/>
+      <c r="C27" s="29"/>
+      <c r="D27" s="29"/>
+      <c r="E27" s="29"/>
+      <c r="F27" s="29"/>
+      <c r="G27" s="29"/>
+      <c r="H27" s="29"/>
+      <c r="I27" s="29"/>
+      <c r="J27" s="29"/>
+      <c r="K27" s="29"/>
+      <c r="L27" s="29"/>
+      <c r="M27" s="29"/>
     </row>
     <row r="29" spans="2:13" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B29" s="36" t="s">
+      <c r="B29" s="37" t="s">
         <v>76</v>
       </c>
-      <c r="C29" s="30"/>
-      <c r="D29" s="30"/>
-      <c r="E29" s="30"/>
-      <c r="F29" s="30"/>
-      <c r="G29" s="30"/>
-      <c r="H29" s="30"/>
-      <c r="I29" s="30"/>
-      <c r="J29" s="30"/>
-      <c r="K29" s="30"/>
-      <c r="L29" s="30"/>
-      <c r="M29" s="30"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="29"/>
+      <c r="F29" s="29"/>
+      <c r="G29" s="29"/>
+      <c r="H29" s="29"/>
+      <c r="I29" s="29"/>
+      <c r="J29" s="29"/>
+      <c r="K29" s="29"/>
+      <c r="L29" s="29"/>
+      <c r="M29" s="29"/>
     </row>
     <row r="30" spans="2:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B30" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="C30" s="34" t="s">
+      <c r="C30" s="35" t="s">
         <v>78</v>
       </c>
-      <c r="D30" s="30"/>
-      <c r="E30" s="30"/>
-      <c r="F30" s="30"/>
-      <c r="G30" s="30"/>
-      <c r="H30" s="30"/>
-      <c r="I30" s="30"/>
-      <c r="J30" s="30"/>
-      <c r="K30" s="30"/>
-      <c r="L30" s="30"/>
-      <c r="M30" s="30"/>
+      <c r="D30" s="29"/>
+      <c r="E30" s="29"/>
+      <c r="F30" s="29"/>
+      <c r="G30" s="29"/>
+      <c r="H30" s="29"/>
+      <c r="I30" s="29"/>
+      <c r="J30" s="29"/>
+      <c r="K30" s="29"/>
+      <c r="L30" s="29"/>
+      <c r="M30" s="29"/>
     </row>
     <row r="31" spans="2:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B31" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="C31" s="34" t="s">
+      <c r="C31" s="35" t="s">
         <v>80</v>
       </c>
-      <c r="D31" s="30"/>
-      <c r="E31" s="30"/>
-      <c r="F31" s="30"/>
-      <c r="G31" s="30"/>
-      <c r="H31" s="30"/>
-      <c r="I31" s="30"/>
-      <c r="J31" s="30"/>
-      <c r="K31" s="30"/>
-      <c r="L31" s="30"/>
-      <c r="M31" s="30"/>
+      <c r="D31" s="29"/>
+      <c r="E31" s="29"/>
+      <c r="F31" s="29"/>
+      <c r="G31" s="29"/>
+      <c r="H31" s="29"/>
+      <c r="I31" s="29"/>
+      <c r="J31" s="29"/>
+      <c r="K31" s="29"/>
+      <c r="L31" s="29"/>
+      <c r="M31" s="29"/>
     </row>
     <row r="32" spans="2:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B32" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="C32" s="34" t="s">
+      <c r="C32" s="35" t="s">
         <v>82</v>
       </c>
-      <c r="D32" s="30"/>
-      <c r="E32" s="30"/>
-      <c r="F32" s="30"/>
-      <c r="G32" s="30"/>
-      <c r="H32" s="30"/>
-      <c r="I32" s="30"/>
-      <c r="J32" s="30"/>
-      <c r="K32" s="30"/>
-      <c r="L32" s="30"/>
-      <c r="M32" s="30"/>
+      <c r="D32" s="29"/>
+      <c r="E32" s="29"/>
+      <c r="F32" s="29"/>
+      <c r="G32" s="29"/>
+      <c r="H32" s="29"/>
+      <c r="I32" s="29"/>
+      <c r="J32" s="29"/>
+      <c r="K32" s="29"/>
+      <c r="L32" s="29"/>
+      <c r="M32" s="29"/>
     </row>
     <row r="33" spans="2:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B33" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="C33" s="34" t="s">
+      <c r="C33" s="35" t="s">
         <v>84</v>
       </c>
-      <c r="D33" s="30"/>
-      <c r="E33" s="30"/>
-      <c r="F33" s="30"/>
-      <c r="G33" s="30"/>
-      <c r="H33" s="30"/>
-      <c r="I33" s="30"/>
-      <c r="J33" s="30"/>
-      <c r="K33" s="30"/>
-      <c r="L33" s="30"/>
-      <c r="M33" s="30"/>
+      <c r="D33" s="29"/>
+      <c r="E33" s="29"/>
+      <c r="F33" s="29"/>
+      <c r="G33" s="29"/>
+      <c r="H33" s="29"/>
+      <c r="I33" s="29"/>
+      <c r="J33" s="29"/>
+      <c r="K33" s="29"/>
+      <c r="L33" s="29"/>
+      <c r="M33" s="29"/>
     </row>
     <row r="34" spans="2:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B34" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="C34" s="34" t="s">
+      <c r="C34" s="35" t="s">
         <v>86</v>
       </c>
-      <c r="D34" s="30"/>
-      <c r="E34" s="30"/>
-      <c r="F34" s="30"/>
-      <c r="G34" s="30"/>
-      <c r="H34" s="30"/>
-      <c r="I34" s="30"/>
-      <c r="J34" s="30"/>
-      <c r="K34" s="30"/>
-      <c r="L34" s="30"/>
-      <c r="M34" s="30"/>
+      <c r="D34" s="29"/>
+      <c r="E34" s="29"/>
+      <c r="F34" s="29"/>
+      <c r="G34" s="29"/>
+      <c r="H34" s="29"/>
+      <c r="I34" s="29"/>
+      <c r="J34" s="29"/>
+      <c r="K34" s="29"/>
+      <c r="L34" s="29"/>
+      <c r="M34" s="29"/>
     </row>
     <row r="35" spans="2:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B35" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="C35" s="34" t="s">
+      <c r="C35" s="35" t="s">
         <v>88</v>
       </c>
-      <c r="D35" s="30"/>
-      <c r="E35" s="30"/>
-      <c r="F35" s="30"/>
-      <c r="G35" s="30"/>
-      <c r="H35" s="30"/>
-      <c r="I35" s="30"/>
-      <c r="J35" s="30"/>
-      <c r="K35" s="30"/>
-      <c r="L35" s="30"/>
-      <c r="M35" s="30"/>
+      <c r="D35" s="29"/>
+      <c r="E35" s="29"/>
+      <c r="F35" s="29"/>
+      <c r="G35" s="29"/>
+      <c r="H35" s="29"/>
+      <c r="I35" s="29"/>
+      <c r="J35" s="29"/>
+      <c r="K35" s="29"/>
+      <c r="L35" s="29"/>
+      <c r="M35" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -2725,28 +2725,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="28" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
     </row>
     <row r="2" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="32" t="s">
         <v>90</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
     </row>
     <row r="3" spans="1:6" ht="8" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B4" s="37" t="s">
+      <c r="B4" s="38" t="s">
         <v>91</v>
       </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
-      <c r="F4" s="30"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="29"/>
+      <c r="F4" s="29"/>
     </row>
     <row r="5" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="6"/>
@@ -2767,13 +2767,13 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B6" s="38" t="s">
+      <c r="B6" s="39" t="s">
         <v>97</v>
       </c>
-      <c r="C6" s="30"/>
-      <c r="D6" s="30"/>
-      <c r="E6" s="30"/>
-      <c r="F6" s="30"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="29"/>
+      <c r="F6" s="29"/>
     </row>
     <row r="7" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B7" s="14" t="s">
@@ -2894,13 +2894,13 @@
       <c r="F14" s="14"/>
     </row>
     <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B15" s="39" t="s">
+      <c r="B15" s="40" t="s">
         <v>117</v>
       </c>
-      <c r="C15" s="30"/>
-      <c r="D15" s="30"/>
-      <c r="E15" s="30"/>
-      <c r="F15" s="30"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="29"/>
     </row>
     <row r="16" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B16" s="7"/>
@@ -3113,13 +3113,13 @@
       <c r="F45" s="10"/>
     </row>
     <row r="46" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B46" s="36" t="s">
+      <c r="B46" s="37" t="s">
         <v>118</v>
       </c>
-      <c r="C46" s="30"/>
-      <c r="D46" s="30"/>
-      <c r="E46" s="30"/>
-      <c r="F46" s="30"/>
+      <c r="C46" s="29"/>
+      <c r="D46" s="29"/>
+      <c r="E46" s="29"/>
+      <c r="F46" s="29"/>
     </row>
     <row r="47" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A47" s="15"/>
@@ -3291,29 +3291,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="28" t="s">
         <v>140</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
     </row>
     <row r="2" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="32" t="s">
         <v>141</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
     </row>
     <row r="3" spans="1:7" ht="8" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="4" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B4" s="41" t="s">
+      <c r="B4" s="42" t="s">
         <v>142</v>
       </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
-      <c r="F4" s="30"/>
-      <c r="G4" s="30"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="29"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
     </row>
     <row r="5" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="6"/>
@@ -3337,14 +3337,14 @@
       </c>
     </row>
     <row r="6" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B6" s="38" t="s">
+      <c r="B6" s="39" t="s">
         <v>149</v>
       </c>
-      <c r="C6" s="30"/>
-      <c r="D6" s="30"/>
-      <c r="E6" s="30"/>
-      <c r="F6" s="30"/>
-      <c r="G6" s="30"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="29"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="29"/>
     </row>
     <row r="7" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B7" s="14" t="s">
@@ -3407,14 +3407,14 @@
       </c>
     </row>
     <row r="10" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B10" s="39" t="s">
+      <c r="B10" s="40" t="s">
         <v>165</v>
       </c>
-      <c r="C10" s="30"/>
-      <c r="D10" s="30"/>
-      <c r="E10" s="30"/>
-      <c r="F10" s="30"/>
-      <c r="G10" s="30"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
     </row>
     <row r="11" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B11" s="7"/>
@@ -3537,14 +3537,14 @@
       <c r="G25" s="9"/>
     </row>
     <row r="27" spans="2:7" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B27" s="40" t="s">
+      <c r="B27" s="41" t="s">
         <v>166</v>
       </c>
-      <c r="C27" s="30"/>
-      <c r="D27" s="30"/>
-      <c r="E27" s="30"/>
-      <c r="F27" s="30"/>
-      <c r="G27" s="30"/>
+      <c r="C27" s="29"/>
+      <c r="D27" s="29"/>
+      <c r="E27" s="29"/>
+      <c r="F27" s="29"/>
+      <c r="G27" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -3580,29 +3580,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="28" t="s">
         <v>167</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
     </row>
     <row r="2" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="32" t="s">
         <v>168</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
     </row>
     <row r="3" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B3" s="45" t="s">
         <v>169</v>
       </c>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
     </row>
     <row r="4" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B4" s="18" t="s">
@@ -3731,12 +3731,12 @@
       <c r="B11" s="45" t="s">
         <v>198</v>
       </c>
-      <c r="C11" s="30"/>
-      <c r="D11" s="30"/>
-      <c r="E11" s="30"/>
-      <c r="F11" s="30"/>
-      <c r="G11" s="30"/>
-      <c r="H11" s="30"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="29"/>
     </row>
     <row r="12" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="15"/>
@@ -3756,14 +3756,14 @@
       <c r="B13" s="20" t="s">
         <v>201</v>
       </c>
-      <c r="C13" s="42" t="s">
+      <c r="C13" s="44" t="s">
         <v>202</v>
       </c>
-      <c r="D13" s="30"/>
-      <c r="E13" s="30"/>
-      <c r="F13" s="30"/>
-      <c r="G13" s="30"/>
-      <c r="H13" s="30"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="29"/>
     </row>
     <row r="14" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B14" s="21" t="s">
@@ -3772,24 +3772,24 @@
       <c r="C14" s="43" t="s">
         <v>204</v>
       </c>
-      <c r="D14" s="30"/>
-      <c r="E14" s="30"/>
-      <c r="F14" s="30"/>
-      <c r="G14" s="30"/>
-      <c r="H14" s="30"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="29"/>
     </row>
     <row r="15" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B15" s="20" t="s">
         <v>205</v>
       </c>
-      <c r="C15" s="42" t="s">
+      <c r="C15" s="44" t="s">
         <v>206</v>
       </c>
-      <c r="D15" s="30"/>
-      <c r="E15" s="30"/>
-      <c r="F15" s="30"/>
-      <c r="G15" s="30"/>
-      <c r="H15" s="30"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="29"/>
+      <c r="H15" s="29"/>
     </row>
     <row r="16" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B16" s="21" t="s">
@@ -3798,24 +3798,24 @@
       <c r="C16" s="43" t="s">
         <v>208</v>
       </c>
-      <c r="D16" s="30"/>
-      <c r="E16" s="30"/>
-      <c r="F16" s="30"/>
-      <c r="G16" s="30"/>
-      <c r="H16" s="30"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="29"/>
+      <c r="H16" s="29"/>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B17" s="20" t="s">
         <v>209</v>
       </c>
-      <c r="C17" s="42" t="s">
+      <c r="C17" s="44" t="s">
         <v>210</v>
       </c>
-      <c r="D17" s="30"/>
-      <c r="E17" s="30"/>
-      <c r="F17" s="30"/>
-      <c r="G17" s="30"/>
-      <c r="H17" s="30"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="29"/>
+      <c r="G17" s="29"/>
+      <c r="H17" s="29"/>
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B18" s="21" t="s">
@@ -3824,24 +3824,24 @@
       <c r="C18" s="43" t="s">
         <v>212</v>
       </c>
-      <c r="D18" s="30"/>
-      <c r="E18" s="30"/>
-      <c r="F18" s="30"/>
-      <c r="G18" s="30"/>
-      <c r="H18" s="30"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="29"/>
+      <c r="H18" s="29"/>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B19" s="20" t="s">
         <v>213</v>
       </c>
-      <c r="C19" s="42" t="s">
+      <c r="C19" s="44" t="s">
         <v>214</v>
       </c>
-      <c r="D19" s="30"/>
-      <c r="E19" s="30"/>
-      <c r="F19" s="30"/>
-      <c r="G19" s="30"/>
-      <c r="H19" s="30"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="29"/>
+      <c r="H19" s="29"/>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B20" s="21" t="s">
@@ -3850,35 +3850,35 @@
       <c r="C20" s="43" t="s">
         <v>216</v>
       </c>
-      <c r="D20" s="30"/>
-      <c r="E20" s="30"/>
-      <c r="F20" s="30"/>
-      <c r="G20" s="30"/>
-      <c r="H20" s="30"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="29"/>
+      <c r="H20" s="29"/>
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B21" s="20" t="s">
         <v>217</v>
       </c>
-      <c r="C21" s="42" t="s">
+      <c r="C21" s="44" t="s">
         <v>218</v>
       </c>
-      <c r="D21" s="30"/>
-      <c r="E21" s="30"/>
-      <c r="F21" s="30"/>
-      <c r="G21" s="30"/>
-      <c r="H21" s="30"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="29"/>
+      <c r="H21" s="29"/>
     </row>
     <row r="23" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B23" s="45" t="s">
         <v>219</v>
       </c>
-      <c r="C23" s="30"/>
-      <c r="D23" s="30"/>
-      <c r="E23" s="30"/>
-      <c r="F23" s="30"/>
-      <c r="G23" s="30"/>
-      <c r="H23" s="30"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="29"/>
+      <c r="F23" s="29"/>
+      <c r="G23" s="29"/>
+      <c r="H23" s="29"/>
     </row>
     <row r="24" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="15"/>
@@ -4070,12 +4070,12 @@
       <c r="B38" s="45" t="s">
         <v>260</v>
       </c>
-      <c r="C38" s="30"/>
-      <c r="D38" s="30"/>
-      <c r="E38" s="30"/>
-      <c r="F38" s="30"/>
-      <c r="G38" s="30"/>
-      <c r="H38" s="30"/>
+      <c r="C38" s="29"/>
+      <c r="D38" s="29"/>
+      <c r="E38" s="29"/>
+      <c r="F38" s="29"/>
+      <c r="G38" s="29"/>
+      <c r="H38" s="29"/>
     </row>
     <row r="39" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A39" s="15"/>
@@ -4098,24 +4098,24 @@
       <c r="C40" s="43" t="s">
         <v>261</v>
       </c>
-      <c r="D40" s="30"/>
-      <c r="E40" s="30"/>
-      <c r="F40" s="30"/>
-      <c r="G40" s="30"/>
-      <c r="H40" s="30"/>
+      <c r="D40" s="29"/>
+      <c r="E40" s="29"/>
+      <c r="F40" s="29"/>
+      <c r="G40" s="29"/>
+      <c r="H40" s="29"/>
     </row>
     <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B41" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="C41" s="42" t="s">
+      <c r="C41" s="44" t="s">
         <v>262</v>
       </c>
-      <c r="D41" s="30"/>
-      <c r="E41" s="30"/>
-      <c r="F41" s="30"/>
-      <c r="G41" s="30"/>
-      <c r="H41" s="30"/>
+      <c r="D41" s="29"/>
+      <c r="E41" s="29"/>
+      <c r="F41" s="29"/>
+      <c r="G41" s="29"/>
+      <c r="H41" s="29"/>
     </row>
     <row r="42" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B42" s="21" t="s">
@@ -4124,24 +4124,24 @@
       <c r="C42" s="43" t="s">
         <v>263</v>
       </c>
-      <c r="D42" s="30"/>
-      <c r="E42" s="30"/>
-      <c r="F42" s="30"/>
-      <c r="G42" s="30"/>
-      <c r="H42" s="30"/>
+      <c r="D42" s="29"/>
+      <c r="E42" s="29"/>
+      <c r="F42" s="29"/>
+      <c r="G42" s="29"/>
+      <c r="H42" s="29"/>
     </row>
     <row r="43" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B43" s="20" t="s">
         <v>128</v>
       </c>
-      <c r="C43" s="42" t="s">
+      <c r="C43" s="44" t="s">
         <v>264</v>
       </c>
-      <c r="D43" s="30"/>
-      <c r="E43" s="30"/>
-      <c r="F43" s="30"/>
-      <c r="G43" s="30"/>
-      <c r="H43" s="30"/>
+      <c r="D43" s="29"/>
+      <c r="E43" s="29"/>
+      <c r="F43" s="29"/>
+      <c r="G43" s="29"/>
+      <c r="H43" s="29"/>
     </row>
     <row r="44" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B44" s="21" t="s">
@@ -4150,24 +4150,24 @@
       <c r="C44" s="43" t="s">
         <v>265</v>
       </c>
-      <c r="D44" s="30"/>
-      <c r="E44" s="30"/>
-      <c r="F44" s="30"/>
-      <c r="G44" s="30"/>
-      <c r="H44" s="30"/>
+      <c r="D44" s="29"/>
+      <c r="E44" s="29"/>
+      <c r="F44" s="29"/>
+      <c r="G44" s="29"/>
+      <c r="H44" s="29"/>
     </row>
     <row r="45" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B45" s="20" t="s">
         <v>104</v>
       </c>
-      <c r="C45" s="42" t="s">
+      <c r="C45" s="44" t="s">
         <v>266</v>
       </c>
-      <c r="D45" s="30"/>
-      <c r="E45" s="30"/>
-      <c r="F45" s="30"/>
-      <c r="G45" s="30"/>
-      <c r="H45" s="30"/>
+      <c r="D45" s="29"/>
+      <c r="E45" s="29"/>
+      <c r="F45" s="29"/>
+      <c r="G45" s="29"/>
+      <c r="H45" s="29"/>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B46" s="21" t="s">
@@ -4176,24 +4176,24 @@
       <c r="C46" s="43" t="s">
         <v>267</v>
       </c>
-      <c r="D46" s="30"/>
-      <c r="E46" s="30"/>
-      <c r="F46" s="30"/>
-      <c r="G46" s="30"/>
-      <c r="H46" s="30"/>
+      <c r="D46" s="29"/>
+      <c r="E46" s="29"/>
+      <c r="F46" s="29"/>
+      <c r="G46" s="29"/>
+      <c r="H46" s="29"/>
     </row>
     <row r="47" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B47" s="20" t="s">
         <v>115</v>
       </c>
-      <c r="C47" s="42" t="s">
+      <c r="C47" s="44" t="s">
         <v>268</v>
       </c>
-      <c r="D47" s="30"/>
-      <c r="E47" s="30"/>
-      <c r="F47" s="30"/>
-      <c r="G47" s="30"/>
-      <c r="H47" s="30"/>
+      <c r="D47" s="29"/>
+      <c r="E47" s="29"/>
+      <c r="F47" s="29"/>
+      <c r="G47" s="29"/>
+      <c r="H47" s="29"/>
     </row>
     <row r="48" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B48" s="21" t="s">
@@ -4202,92 +4202,92 @@
       <c r="C48" s="43" t="s">
         <v>269</v>
       </c>
-      <c r="D48" s="30"/>
-      <c r="E48" s="30"/>
-      <c r="F48" s="30"/>
-      <c r="G48" s="30"/>
-      <c r="H48" s="30"/>
+      <c r="D48" s="29"/>
+      <c r="E48" s="29"/>
+      <c r="F48" s="29"/>
+      <c r="G48" s="29"/>
+      <c r="H48" s="29"/>
     </row>
     <row r="50" spans="2:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B50" s="45" t="s">
         <v>270</v>
       </c>
-      <c r="C50" s="30"/>
-      <c r="D50" s="30"/>
-      <c r="E50" s="30"/>
-      <c r="F50" s="30"/>
-      <c r="G50" s="30"/>
-      <c r="H50" s="30"/>
+      <c r="C50" s="29"/>
+      <c r="D50" s="29"/>
+      <c r="E50" s="29"/>
+      <c r="F50" s="29"/>
+      <c r="G50" s="29"/>
+      <c r="H50" s="29"/>
     </row>
     <row r="51" spans="2:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B51" s="24" t="s">
         <v>100</v>
       </c>
-      <c r="C51" s="44" t="s">
+      <c r="C51" s="47" t="s">
         <v>271</v>
       </c>
-      <c r="D51" s="30"/>
-      <c r="E51" s="30"/>
-      <c r="F51" s="30"/>
-      <c r="G51" s="30"/>
-      <c r="H51" s="30"/>
+      <c r="D51" s="29"/>
+      <c r="E51" s="29"/>
+      <c r="F51" s="29"/>
+      <c r="G51" s="29"/>
+      <c r="H51" s="29"/>
     </row>
     <row r="52" spans="2:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B52" s="25" t="s">
         <v>106</v>
       </c>
-      <c r="C52" s="46" t="s">
+      <c r="C52" s="48" t="s">
         <v>272</v>
       </c>
-      <c r="D52" s="30"/>
-      <c r="E52" s="30"/>
-      <c r="F52" s="30"/>
-      <c r="G52" s="30"/>
-      <c r="H52" s="30"/>
+      <c r="D52" s="29"/>
+      <c r="E52" s="29"/>
+      <c r="F52" s="29"/>
+      <c r="G52" s="29"/>
+      <c r="H52" s="29"/>
     </row>
     <row r="53" spans="2:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B53" s="26" t="s">
         <v>273</v>
       </c>
-      <c r="C53" s="47" t="s">
+      <c r="C53" s="46" t="s">
         <v>274</v>
       </c>
-      <c r="D53" s="30"/>
-      <c r="E53" s="30"/>
-      <c r="F53" s="30"/>
-      <c r="G53" s="30"/>
-      <c r="H53" s="30"/>
+      <c r="D53" s="29"/>
+      <c r="E53" s="29"/>
+      <c r="F53" s="29"/>
+      <c r="G53" s="29"/>
+      <c r="H53" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="C14:H14"/>
-    <mergeCell ref="C45:H45"/>
-    <mergeCell ref="B38:H38"/>
-    <mergeCell ref="C20:H20"/>
+    <mergeCell ref="C47:H47"/>
+    <mergeCell ref="C44:H44"/>
+    <mergeCell ref="C40:H40"/>
+    <mergeCell ref="C43:H43"/>
+    <mergeCell ref="C21:H21"/>
     <mergeCell ref="C53:H53"/>
     <mergeCell ref="C18:H18"/>
     <mergeCell ref="B11:H11"/>
     <mergeCell ref="B23:H23"/>
     <mergeCell ref="C15:H15"/>
     <mergeCell ref="C42:H42"/>
-    <mergeCell ref="A2:C2"/>
     <mergeCell ref="C51:H51"/>
     <mergeCell ref="C46:H46"/>
     <mergeCell ref="B50:H50"/>
     <mergeCell ref="C52:H52"/>
     <mergeCell ref="C48:H48"/>
     <mergeCell ref="C17:H17"/>
-    <mergeCell ref="B3:H3"/>
     <mergeCell ref="C19:H19"/>
     <mergeCell ref="C13:H13"/>
     <mergeCell ref="C41:H41"/>
     <mergeCell ref="C16:H16"/>
-    <mergeCell ref="C47:H47"/>
-    <mergeCell ref="C44:H44"/>
-    <mergeCell ref="C40:H40"/>
-    <mergeCell ref="C43:H43"/>
-    <mergeCell ref="C21:H21"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="C14:H14"/>
+    <mergeCell ref="C45:H45"/>
+    <mergeCell ref="B38:H38"/>
+    <mergeCell ref="C20:H20"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="B3:H3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>

</xml_diff>